<commit_message>
Density categories (<10^4, 10^4, 10^5, >10^5) in sample_metadata.csv; CFU analysis by category; Supplementary Tables 1 and 6 regenerated
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/supplement/Supplementary_Tables.xlsx
+++ b/results/supplement/Supplementary_Tables.xlsx
@@ -461,7 +461,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LAMP result: 1 = positive (uidA: &lt;= 30 min and &gt;= 3-fold; papGII: &lt;= 23 min and &gt;= 3-fold); time to threshold empty = fluorescence threshold not reached within 40 min. Bacterial density from semi-quantitative culture of 10 ul; the category 10^5 includes &gt;10^5 CFU/ml. papG alleles: BLASTN vs papG classes I-IV (&gt;= 90% identity, &gt;= 80% coverage); phylogroups: EzClermont.</t>
+          <t>LAMP result: 1 = positive (uidA: &lt;= 30 min and &gt;= 3-fold; papGII: &lt;= 23 min and &gt;= 3-fold); time to threshold empty = fluorescence threshold not reached within 40 min. Bacterial density from semi-quantitative culture of 10 ul (categories &lt;10^4, 10^4, 10^5 and &gt;10^5 CFU/ml). papG alleles: BLASTN vs papG classes I-IV (&gt;= 90% identity, &gt;= 80% coverage); phylogroups: EzClermont.</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1829,7 +1829,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>10^4</t>
+          <t>&lt;10^4</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2613,7 +2613,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>10^4</t>
+          <t>&lt;10^4</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3351,7 +3351,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -3647,7 +3647,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -3703,7 +3703,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3749,7 +3749,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3949,7 +3949,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>10^4</t>
+          <t>&lt;10^4</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -4041,7 +4041,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -4087,7 +4087,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -4145,7 +4145,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -4953,7 +4953,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>10^4</t>
+          <t>&lt;10^4</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -5395,7 +5395,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5693,7 +5693,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -5839,7 +5839,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -5939,7 +5939,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -6037,7 +6037,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -6095,7 +6095,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -6635,7 +6635,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -6681,7 +6681,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -6737,7 +6737,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -7023,7 +7023,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -7399,7 +7399,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -7685,7 +7685,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -7779,7 +7779,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -7873,7 +7873,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -7919,7 +7919,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -7965,7 +7965,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -8057,7 +8057,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -8113,7 +8113,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -8169,7 +8169,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -8225,7 +8225,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -8281,7 +8281,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -8579,7 +8579,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -8625,7 +8625,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -9011,7 +9011,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -9069,7 +9069,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -9461,7 +9461,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -9517,7 +9517,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -9575,7 +9575,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -9947,7 +9947,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -13807,7 +13807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -13879,7 +13879,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -13937,7 +13937,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -13966,7 +13966,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -13995,7 +13995,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -14024,7 +14024,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -14051,7 +14051,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -14078,7 +14078,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -14105,7 +14105,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -14134,7 +14134,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -14161,7 +14161,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -14188,7 +14188,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -14217,7 +14217,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -14244,7 +14244,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -14273,7 +14273,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -14302,7 +14302,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -14331,7 +14331,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -14358,7 +14358,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -14385,7 +14385,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -14412,7 +14412,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -14439,7 +14439,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -14466,7 +14466,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -14495,7 +14495,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -14522,7 +14522,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -14551,7 +14551,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -14578,7 +14578,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -14605,7 +14605,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -14634,7 +14634,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -14661,7 +14661,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -14773,7 +14773,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -14800,7 +14800,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -14856,7 +14856,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -14883,7 +14883,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>&gt;10^5</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -14912,7 +14912,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>10^5 (includes &gt;10^5)</t>
+          <t>10^5</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -14970,131 +14970,166 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2. uidA TTT by papGII status</t>
+          <t xml:space="preserve">  category 10^4: n=4 median=28.5 IQR=25.0-29.2 range=16-30 never_crossed=0; papGII-positive: 0</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">  all loads: papGII+ n=6 median=21.0 IQR=18.8-24.8 range=18-26 never_crossed=0</t>
+          <t xml:space="preserve">  category 10^5: n=7 median=27.5 IQR=26.2-29.5 range=21-33 never_crossed=1; papGII-positive: 1</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">  all loads: papGII- n=32 median=24.0 IQR=19.5-28.0 range=14-36 never_crossed=1</t>
+          <t xml:space="preserve">  category &gt;10^5: n=27 median=21.0 IQR=18.5-26.0 range=14-36 never_crossed=0; papGII-positive: 5</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">  all loads: Mann-Whitney p = 0.273</t>
+          <t xml:space="preserve">  &gt;10^5 vs &lt;=10^5 CFU/ml: n=27 median=21.0 IQR=18.5-26.0 range=14-36 never_crossed=0 vs n=11 median=28.0 IQR=26.2-29.8 range=16-33 never_crossed=1; Mann-Whitney p = 0.028</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;=10^5 CFU/ml: papGII+ n=6 median=21.0 IQR=18.8-24.8 range=18-26 never_crossed=0</t>
+          <t xml:space="preserve">  within &gt;10^5 CFU/ml: papGII+ n=5 median=21.0 IQR=18.0-26.0 range=18-26 never_crossed=0 vs papGII- n=22 median=21.5 IQR=19.0-25.8 range=14-36 never_crossed=0; Mann-Whitney p = 0.729</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;=10^5 CFU/ml: papGII- n=28 median=22.0 IQR=19.5-27.5 range=14-36 never_crossed=1</t>
+          <t>2. uidA TTT by papGII status</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">  &gt;=10^5 CFU/ml: Mann-Whitney p = 0.336</t>
+          <t xml:space="preserve">  all loads: papGII+ n=6 median=21.0 IQR=18.8-24.8 range=18-26 never_crossed=0</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>3. papGII vs uidA primer set in papGII-positive urines (paired)</t>
+          <t xml:space="preserve">  all loads: papGII- n=32 median=24.0 IQR=19.5-28.0 range=14-36 never_crossed=1</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">  papGII primers: n=6 median=17.0 IQR=16.0-18.0 range=13-20 never_crossed=0</t>
+          <t xml:space="preserve">  all loads: Mann-Whitney p = 0.273</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">  uidA primers:   n=6 median=21.0 IQR=18.8-24.8 range=18-26 never_crossed=0</t>
+          <t xml:space="preserve">  &gt;=10^5 CFU/ml: papGII+ n=6 median=21.0 IQR=18.8-24.8 range=18-26 never_crossed=0</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">  papGII earlier in 6/6; median difference 5.0 min; exact Wilcoxon p = 0.031</t>
+          <t xml:space="preserve">  &gt;=10^5 CFU/ml: papGII- n=28 median=22.0 IQR=19.5-27.5 range=14-36 never_crossed=1</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>4. uidA TTT in mixed vs single-species cultures</t>
+          <t xml:space="preserve">  &gt;=10^5 CFU/ml: Mann-Whitney p = 0.336</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">  mixed: n=5 median=28.0 IQR=27.0-34.0 range=19-35 never_crossed=0</t>
+          <t>3. papGII vs uidA primer set in papGII-positive urines (paired)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">  single: n=33 median=22.0 IQR=18.8-26.2 range=14-36 never_crossed=1</t>
+          <t xml:space="preserve">  papGII primers: n=6 median=17.0 IQR=16.0-18.0 range=13-20 never_crossed=0</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>5. TTT of reference-positive vs reference-negative samples</t>
+          <t xml:space="preserve">  uidA primers:   n=6 median=21.0 IQR=18.8-24.8 range=18-26 never_crossed=0</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">  uidA positives: n=38 median=22.0 IQR=19.0-28.0 range=14-36 never_crossed=1</t>
+          <t xml:space="preserve">  papGII earlier in 6/6; median difference 5.0 min; exact Wilcoxon p = 0.031</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">  uidA negatives crossing: n=153 median=34.0 IQR=32.0-38.0 range=18-40 never_crossed=91; earliest 18 min; crossing after the 30-min threshold: 54</t>
+          <t>4. uidA TTT in mixed vs single-species cultures</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">  papGII positives: n=6 median=17.0 IQR=16.0-18.0 range=13-20 never_crossed=0</t>
+          <t xml:space="preserve">  mixed: n=5 median=28.0 IQR=27.0-34.0 range=19-35 never_crossed=0</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  single: n=33 median=22.0 IQR=18.8-26.2 range=14-36 never_crossed=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>5. TTT of reference-positive vs reference-negative samples</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  uidA positives: n=38 median=22.0 IQR=19.0-28.0 range=14-36 never_crossed=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  uidA negatives crossing: n=153 median=34.0 IQR=32.0-38.0 range=18-40 never_crossed=91; earliest 18 min; crossing after the 30-min threshold: 54</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  papGII positives: n=6 median=17.0 IQR=16.0-18.0 range=13-20 never_crossed=0</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
         <is>
           <t xml:space="preserve">  papGII negatives crossing: n=185 median=35.0 IQR=32.0-38.0 range=26-40 never_crossed=112; earliest 26 min; crossing after the 23-min threshold: 73</t>
         </is>

</xml_diff>